<commit_message>
🤖 Atualização Automática: Dados IPMA
</commit_message>
<xml_diff>
--- a/Painel_Mestre_IPMA.xlsx
+++ b/Painel_Mestre_IPMA.xlsx
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1464,7 +1464,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1699,7 +1699,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>

</xml_diff>